<commit_message>
Add category breakdown, category chart, and overweight positions table (>5%)
</commit_message>
<xml_diff>
--- a/data/base_de_donnees.xlsx
+++ b/data/base_de_donnees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/52abc88aebc4debd/Documents/Quintet/HealthCheck/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{95AE71BE-2A97-4BBF-AC2D-F077D52D3990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3149DC9-3733-4915-BB19-B917CE488BF6}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="8_{95AE71BE-2A97-4BBF-AC2D-F077D52D3990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3D8E213-B3C3-4532-A75B-8C99571202C9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AB568F40-28DD-4332-8525-8E1108A9606E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="25">
   <si>
     <t>ISIN</t>
   </si>
@@ -90,6 +90,30 @@
   </si>
   <si>
     <t>USD</t>
+  </si>
+  <si>
+    <t>Catégorie</t>
+  </si>
+  <si>
+    <t>Equity</t>
+  </si>
+  <si>
+    <t>Fixed Income</t>
+  </si>
+  <si>
+    <t>CS FI10</t>
+  </si>
+  <si>
+    <t>CHF</t>
+  </si>
+  <si>
+    <t>CHF5646569</t>
+  </si>
+  <si>
+    <t>CHF7868</t>
+  </si>
+  <si>
+    <t>Nestlé</t>
   </si>
 </sst>
 </file>
@@ -462,7 +486,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32D3F8D0-2983-4485-B560-E3840825A905}">
-  <dimension ref="C2:H6"/>
+  <dimension ref="C2:H8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="3:8" x14ac:dyDescent="0.3">
@@ -481,6 +505,9 @@
       <c r="G2" t="s">
         <v>7</v>
       </c>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="3" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
@@ -498,7 +525,9 @@
       <c r="G3" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="1"/>
+      <c r="H3" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="4" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
@@ -516,7 +545,9 @@
       <c r="G4" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="1"/>
+      <c r="H4" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="5" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
@@ -529,12 +560,14 @@
         <v>2</v>
       </c>
       <c r="F5" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="1"/>
+      <c r="H5" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="6" spans="3:8" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
@@ -551,6 +584,46 @@
       </c>
       <c r="G6" t="s">
         <v>13</v>
+      </c>
+      <c r="H6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7">
+        <v>200</v>
+      </c>
+      <c r="F7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" t="s">
+        <v>8</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8">
+        <v>55</v>
+      </c>
+      <c r="F8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>